<commit_message>
Enhanced slides with graphics and better bullet style
</commit_message>
<xml_diff>
--- a/SOL M5.xlsx
+++ b/SOL M5.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\QA\Software Craft - ADXD2SD4M5\2025 new course\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\QA\2025 M5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2871F800-CF82-44A6-A842-FE1227EE6424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{722CDE27-3D68-489B-9196-D9D583D0FD3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -265,6 +265,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFF6F8FC"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -274,6 +279,270 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>106680</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>548640</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>68580</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{42A67B8F-333B-35AE-9A7A-55ED7CA6FC05}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6957060" y="266700"/>
+          <a:ext cx="7147560" cy="4373880"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="F6F8FC"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>Knowledge</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>K7:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t> software design approaches and patterns, to identify reusable solutions to commonly occurring problems</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="1000" b="1"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>K8:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t> organisational policies and procedures relating to the tasks being undertaken, and when to follow them. </a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-GB" sz="1000"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t>	For example, the storage and treatment of GDPR sensitive data.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>K11</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t> software designs and functional/technical specifications.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>K12:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t> software testing frameworks and methodologies</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-GB" sz="1000"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>Skills</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>S4:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t> test code and analyse results to correct errors found using unit testing</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>S6:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t> identify and create test scenarios</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>S7:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t> apply structured techniques to problem solving, can debug code and can understand the structure of programmes to identify and resolve issues </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>S9:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t> create analysis artefacts, such as use cases and/or user stories</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>S12:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t> follow software designs and functional/technical specifications</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>S17:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t> interpret and implement a given design whist remaining compliant with security and maintainability requirements</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-GB" sz="1000"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>Behaviours</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>B1:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t> Works independently and takes responsibility. For example, has a disciplined and responsible approach to risk, </a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-GB" sz="1000"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t>and stays motivated and committed when facing challenges</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-GB" sz="1000"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>B2:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t> Applies logical thinking. For example, uses clear and valid reasoning when making decisions related to undertaking work instructions.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>B3:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t> Maintains a productive, professional and secure working environment</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>B5:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t> Acts with integrity with respect to ethical, legal and regulatory ensuring the protection of personal data, safety and security.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000" b="1"/>
+            <a:t>B6:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1000"/>
+            <a:t> Shows initiative for solving problems within their own remit being resourceful when faced with a problem to solve.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-GB" sz="1000"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1240,6 +1509,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>